<commit_message>
S1: correct section reference, American spelling in labels; README: point to docs/supplementary
</commit_message>
<xml_diff>
--- a/docs/supplementary/Supplementary_Table_S1_included_studies.xlsx
+++ b/docs/supplementary/Supplementary_Table_S1_included_studies.xlsx
@@ -57,7 +57,7 @@
     <t xml:space="preserve">Modality</t>
   </si>
   <si>
-    <t xml:space="preserve">Ionising modality</t>
+    <t xml:space="preserve">Ionizing modality</t>
   </si>
   <si>
     <t xml:space="preserve">Quantum paradigm</t>
@@ -78,7 +78,7 @@
     <t xml:space="preserve">Classical baseline</t>
   </si>
   <si>
-    <t xml:space="preserve">Baseline rigour</t>
+    <t xml:space="preserve">Baseline rigor</t>
   </si>
   <si>
     <t xml:space="preserve">Statistical testing</t>
@@ -225,7 +225,7 @@
     <t xml:space="preserve">3 and 4 qubits (8 and 16 features); executed on the 21-qubit IonQ Aria</t>
   </si>
   <si>
-    <t xml:space="preserve">Private single-centre</t>
+    <t xml:space="preserve">Private single-center</t>
   </si>
   <si>
     <t xml:space="preserve">Code without model weights</t>
@@ -309,7 +309,7 @@
     <t xml:space="preserve">Lebanon</t>
   </si>
   <si>
-    <t xml:space="preserve">Private multi-centre</t>
+    <t xml:space="preserve">Private multi-center</t>
   </si>
   <si>
     <t xml:space="preserve">10.1007/s10278-025-01630-3</t>
@@ -2037,7 +2037,7 @@
     <t xml:space="preserve">All characteristics are copied from the committed extraction workbook 7-Manuscript/supp_enrich/out/extractions_ai_enriched_v134.xlsx in the public repository https://github.com/lpapp-muw/qc-medimaging-review, restricted to the 133 included studies (the workbook also holds the study excluded during the critical appraisal). Values were extracted by AI with verbatim-quote grounding and derived by deterministic scripts, as described in Sections II-E to II-G of the manuscript. Nothing was re-extracted for this table.</t>
   </si>
   <si>
-    <t xml:space="preserve">Dataset realism applies the post-appraisal correction overlay 7-Manuscript/provenance/extraction_corrections_post_appraisal.json (two studies, one moved from single-centre to multi-centre and one in the opposite direction).</t>
+    <t xml:space="preserve">Dataset realism applies the post-appraisal correction overlay 7-Manuscript/provenance/extraction_corrections_post_appraisal.json (two studies, one moved from single-center to multi-center and one in the opposite direction).</t>
   </si>
   <si>
     <t xml:space="preserve">Publication year is taken from the co-author extraction (6-InterRaterKappa/human.xlsx), because the AI workbook does not carry it. Country names are merged for spelling variants only (for example Republic of Korea and South Korea).</t>
@@ -2061,7 +2061,7 @@
     <t xml:space="preserve">Clinical-readiness and resource-accounting scores are defined in Section II-H. The resource-accounting score counts quantities reported in the main text.</t>
   </si>
   <si>
-    <t xml:space="preserve">Quality-fit subset marks the seven studies meeting the pre-registered sensitivity criteria (Section III-J).</t>
+    <t xml:space="preserve">Quality-fit subset marks the seven studies meeting the pre-registered sensitivity criteria (Section III-H).</t>
   </si>
   <si>
     <t xml:space="preserve">Quantity</t>
@@ -2100,7 +2100,7 @@
     <t xml:space="preserve">Classical baseline present</t>
   </si>
   <si>
-    <t xml:space="preserve">Strictest baseline rigour</t>
+    <t xml:space="preserve">Strictest baseline rigor</t>
   </si>
   <si>
     <t xml:space="preserve">Reproducibility tier none</t>

</xml_diff>